<commit_message>
docs: add Campeon sheet and update Ranking formulas with sum of champion points
</commit_message>
<xml_diff>
--- a/puntos.xlsx
+++ b/puntos.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
     <sheet name="Pronósticos" sheetId="2" r:id="rId2"/>
+    <sheet name="Campeón" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -448,7 +449,7 @@
         <v>Ulises Saul Ramirez Diaz</v>
       </c>
       <c r="C5">
-        <f>SUM(Pronósticos!AR$4:AR$108)</f>
+        <f>SUM(Pronósticos!AR$4:AR$107)+Campeón!E2</f>
         <v>232</v>
       </c>
       <c r="D5">
@@ -478,7 +479,7 @@
         <v>Gabriel Maldonado</v>
       </c>
       <c r="C6">
-        <f>SUM(Pronósticos!T$4:T$108)</f>
+        <f>SUM(Pronósticos!T$4:T$107)+Campeón!E3</f>
         <v>224</v>
       </c>
       <c r="D6">
@@ -508,7 +509,7 @@
         <v>Rodrigo Esteban</v>
       </c>
       <c r="C7">
-        <f>SUM(Pronósticos!AL$4:AL$108)</f>
+        <f>SUM(Pronósticos!AL$4:AL$107)+Campeón!E4</f>
         <v>223</v>
       </c>
       <c r="D7">
@@ -538,7 +539,7 @@
         <v>Jorge Galaviz</v>
       </c>
       <c r="C8">
-        <f>SUM(Pronósticos!AD$4:AD$108)</f>
+        <f>SUM(Pronósticos!AD$4:AD$107)+Campeón!E5</f>
         <v>214</v>
       </c>
       <c r="D8">
@@ -568,7 +569,7 @@
         <v>Juan Pablo</v>
       </c>
       <c r="C9">
-        <f>SUM(Pronósticos!AF$4:AF$108)</f>
+        <f>SUM(Pronósticos!AF$4:AF$107)+Campeón!E6</f>
         <v>213</v>
       </c>
       <c r="D9">
@@ -598,7 +599,7 @@
         <v>Roberto Bautista Eleuterio</v>
       </c>
       <c r="C10">
-        <f>SUM(Pronósticos!AJ$4:AJ$108)</f>
+        <f>SUM(Pronósticos!AJ$4:AJ$107)+Campeón!E7</f>
         <v>212</v>
       </c>
       <c r="D10">
@@ -628,7 +629,7 @@
         <v>Alfredo</v>
       </c>
       <c r="C11">
-        <f>SUM(Pronósticos!L$4:L$108)</f>
+        <f>SUM(Pronósticos!L$4:L$107)+Campeón!E8</f>
         <v>207</v>
       </c>
       <c r="D11">
@@ -658,7 +659,7 @@
         <v>Mau7</v>
       </c>
       <c r="C12">
-        <f>SUM(Pronósticos!AH$4:AH$108)</f>
+        <f>SUM(Pronósticos!AH$4:AH$107)+Campeón!E9</f>
         <v>200</v>
       </c>
       <c r="D12">
@@ -688,7 +689,7 @@
         <v>Joel Garcia</v>
       </c>
       <c r="C13">
-        <f>SUM(Pronósticos!AB$4:AB$108)</f>
+        <f>SUM(Pronósticos!AB$4:AB$107)+Campeón!E10</f>
         <v>199</v>
       </c>
       <c r="D13">
@@ -718,7 +719,7 @@
         <v>Cachorro Zamora</v>
       </c>
       <c r="C14">
-        <f>SUM(Pronósticos!N$4:N$108)</f>
+        <f>SUM(Pronósticos!N$4:N$107)+Campeón!E11</f>
         <v>198</v>
       </c>
       <c r="D14">
@@ -748,7 +749,7 @@
         <v>Rodrigo Morales</v>
       </c>
       <c r="C15">
-        <f>SUM(Pronósticos!AN$4:AN$108)</f>
+        <f>SUM(Pronósticos!AN$4:AN$107)+Campeón!E12</f>
         <v>196</v>
       </c>
       <c r="D15">
@@ -778,7 +779,7 @@
         <v>Eugenio</v>
       </c>
       <c r="C16">
-        <f>SUM(Pronósticos!R$4:R$108)</f>
+        <f>SUM(Pronósticos!R$4:R$107)+Campeón!E13</f>
         <v>192</v>
       </c>
       <c r="D16">
@@ -808,7 +809,7 @@
         <v>CR666</v>
       </c>
       <c r="C17">
-        <f>SUM(Pronósticos!P$4:P$108)</f>
+        <f>SUM(Pronósticos!P$4:P$107)+Campeón!E14</f>
         <v>189</v>
       </c>
       <c r="D17">
@@ -838,7 +839,7 @@
         <v>GERMAN JUAREZ ARIAS</v>
       </c>
       <c r="C18">
-        <f>SUM(Pronósticos!V$4:V$108)</f>
+        <f>SUM(Pronósticos!V$4:V$107)+Campeón!E15</f>
         <v>187</v>
       </c>
       <c r="D18">
@@ -868,7 +869,7 @@
         <v>jmc</v>
       </c>
       <c r="C19">
-        <f>SUM(Pronósticos!Z$4:Z$108)</f>
+        <f>SUM(Pronósticos!Z$4:Z$107)+Campeón!E16</f>
         <v>163</v>
       </c>
       <c r="D19">
@@ -898,7 +899,7 @@
         <v>Salvador19890903</v>
       </c>
       <c r="C20">
-        <f>SUM(Pronósticos!AP$4:AP$108)</f>
+        <f>SUM(Pronósticos!AP$4:AP$107)+Campeón!E17</f>
         <v>117</v>
       </c>
       <c r="D20">
@@ -928,7 +929,7 @@
         <v>Javier</v>
       </c>
       <c r="C21">
-        <f>SUM(Pronósticos!X$4:X$108)</f>
+        <f>SUM(Pronósticos!X$4:X$107)+Campeón!E18</f>
         <v>106</v>
       </c>
       <c r="D21">
@@ -4911,7 +4912,7 @@
         <v>5</v>
       </c>
       <c r="U32" t="str">
-        <v>undefined-0</v>
+        <v>2-0</v>
       </c>
       <c r="V32">
         <v>5</v>
@@ -7281,7 +7282,7 @@
         <v>3</v>
       </c>
       <c r="Y50" t="str">
-        <v>3-0</v>
+        <v>undefined-0</v>
       </c>
       <c r="Z50">
         <v>3</v>
@@ -11330,7 +11331,7 @@
         <v>3</v>
       </c>
       <c r="U81" t="str">
-        <v>1-2</v>
+        <v>undefined-2</v>
       </c>
       <c r="V81">
         <v>5</v>
@@ -14827,4 +14828,321 @@
     <ignoredError numberStoredAsText="1" sqref="A1:AR107"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E18"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Participante</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Predicción Campeón</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Goles Local</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Goles Visitante</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Puntos</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Ulises Saul Ramirez Diaz</v>
+      </c>
+      <c r="B2" t="str">
+        <v>España</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Gabriel Maldonado</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Rodrigo Esteban</v>
+      </c>
+      <c r="B4" t="str">
+        <v>España</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>2</v>
+      </c>
+      <c r="E4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Jorge Galaviz</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Portugal</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Juan Pablo</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Argentina</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Roberto Bautista Eleuterio</v>
+      </c>
+      <c r="B7" t="str">
+        <v>España</v>
+      </c>
+      <c r="C7">
+        <v>3</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Alfredo</v>
+      </c>
+      <c r="B8" t="str">
+        <v>España</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Mau7</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Joel Garcia</v>
+      </c>
+      <c r="B10" t="str">
+        <v>España</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Cachorro Zamora</v>
+      </c>
+      <c r="B11" t="str">
+        <v>España</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Rodrigo Morales</v>
+      </c>
+      <c r="B12" t="str">
+        <v>España</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Eugenio</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>CR666</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Países Bajos</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>GERMAN JUAREZ ARIAS</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Francia</v>
+      </c>
+      <c r="C15">
+        <v>2</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>jmc</v>
+      </c>
+      <c r="B16" t="str">
+        <v>-</v>
+      </c>
+      <c r="C16" t="str">
+        <v>-</v>
+      </c>
+      <c r="D16" t="str">
+        <v>-</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Salvador19890903</v>
+      </c>
+      <c r="B17" t="str">
+        <v>España</v>
+      </c>
+      <c r="C17">
+        <v>2</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Javier</v>
+      </c>
+      <c r="B18" t="str">
+        <v>España</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E18"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>